<commit_message>
studied and applied different charts to different data
</commit_message>
<xml_diff>
--- a/Logical Functions.xlsx
+++ b/Logical Functions.xlsx
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="58">
   <si>
     <t>Full Name</t>
   </si>
@@ -202,6 +202,12 @@
   </si>
   <si>
     <t>LOOKUP</t>
+  </si>
+  <si>
+    <t>SUMIF</t>
+  </si>
+  <si>
+    <t>SUMIFS</t>
   </si>
   <si>
     <t>HLOOKUP</t>
@@ -232,7 +238,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -266,13 +272,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF00B0F0"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -836,152 +835,152 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1055,6 +1054,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1440,7 +1441,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:U26"/>
+  <dimension ref="A1:U24"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="13.7777777777778" customWidth="1"/>
@@ -1995,14 +1996,26 @@
       <c r="M15" s="17"/>
       <c r="N15" s="17"/>
     </row>
-    <row r="24" spans="6:21">
-      <c r="U24" s="29"/>
-    </row>
-    <row r="26" spans="6:21">
-      <c r="F26" t="e">
-        <f>l</f>
-        <v>#NAME?</v>
-      </c>
+    <row r="21" spans="7:21">
+      <c r="G21" s="29" t="s">
+        <v>50</v>
+      </c>
+      <c r="H21" s="30">
+        <f>SUMIF(B2:B9,"marathi",C2:C9)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="7:21">
+      <c r="G22" s="29" t="s">
+        <v>51</v>
+      </c>
+      <c r="H22" s="30">
+        <f>SUMIFS(C2:C9,B2:B9,"English",F2:F9,"Average Marks")</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="24" spans="7:21">
+      <c r="U24" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2031,7 +2044,7 @@
   <sheetData>
     <row r="1" ht="15.6" spans="1:11">
       <c r="A1" s="10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -2166,12 +2179,12 @@
         <v>36</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="16" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B7" s="9" t="str">
         <f>HLOOKUP(B6,A2:K4,3,FALSE)</f>
@@ -2290,7 +2303,7 @@
         <v>895</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E5" s="5"/>
       <c r="F5" s="6"/>
@@ -2326,7 +2339,7 @@
         <v>783</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E7" s="9" t="str">
         <f>VLOOKUP(D7,A1:C11,2,FALSE)</f>
@@ -2339,7 +2352,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>29</v>
@@ -2454,7 +2467,7 @@
         <v>895</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E5" s="5"/>
       <c r="F5" s="6"/>
@@ -2503,7 +2516,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>29</v>
@@ -2555,11 +2568,11 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<DataMashup xmlns="http://schemas.microsoft.com/DataMashup">AAAAAGwDAABQSwMECgAAAAAAh07iQAAAAAAAAAAAAAAAAAcAAABDb25maWcvUEsDBBQAAAAIAIdO4kASOP6YnwAAAPMAAAASAAAAQ29uZmlnL1BhY2thZ2UueG1shY9NC4IwHMa/iuzuNmdRyN958JoRBNF1zDVHOsPNJn36jDK6dXtefofngWLq2uiuBmd6m6MEUxQpK/vaWJ2j0V/iLSo4HIS8Cq2iGbYum1ydo8b7W0ZICAGHFPeDJozShJyr3VE2qhPoC5v/cGys88JKhTic3mM4w8lqg9N1iimQJYTK2EUzzOa9r/YnhHJs/Tgo/mjicg9ksUA+H/gTUEsDBAoAAAAAAIdO4kAAAAAAAAAAAAAAAAAJAAAARm9ybXVsYXMvUEsDBBQAAAAIAIdO4kAoike4DgAAABEAAAATAAAARm9ybXVsYXMvU2VjdGlvbjEubStOTS7JzM9TCIbQhtYAUEsDBBQAAAAIAIdO4kB/v9PKnQAAAOQAAAATAAAAW0NvbnRlbnRfVHlwZXNdLnhtbG2PSw7CMAxErxJ5n7qwQAg17aJwAy4QBfcjmo8aF4Xbk9AdYunxPM+46ZJdxIvWOHun4FDVIMgZ/5jdqGDjQZ6ha5v7O1AU2eqigok5XBCjmcjqWPlALm8Gv1rNeVxHDNo89Uh4rOsTGu+YHEsuN6BtrjTobWFxS1neYzMOot99JUoBU2IsMv4F7I9dh7DMRnN+ApO0UdoC4rd2+wFQSwECFAAUAAAACACHTuJAf7/Typ0AAADkAAAAEwAAAAAAAAABACAAAABaAQAAW0NvbnRlbnRfVHlwZXNdLnhtbFBLAQIUAAoAAAAAAIdO4kAAAAAAAAAAAAAAAAAHAAAAAAAAAAAAEAAAAAAAAABDb25maWcvUEsBAhQAFAAAAAgAh07iQBI4/pifAAAA8wAAABIAAAAAAAAAAQAgAAAAJQAAAENvbmZpZy9QYWNrYWdlLnhtbFBLAQIUAAoAAAAAAIdO4kAAAAAAAAAAAAAAAAAJAAAAAAAAAAAAEAAAAPQAAABGb3JtdWxhcy9QSwECFAAUAAAACACHTuJAKIpHuA4AAAARAAAAEwAAAAAAAAABACAAAAAbAQAARm9ybXVsYXMvU2VjdGlvbjEubVBLBQYAAAAABQAFAC4BAAAoAgAAAAAOAQAAPD94bWwgdmVyc2lvbj0iMS4wIiBlbmNvZGluZz0idXRmLTgiID8+PFBlcm1pc3Npb25MaXN0IHhtbG5zOnhzZD0iaHR0cDovL3d3dy53My5vcmcvMjAwMS9YTUxTY2hlbWEiIHhtbG5zOnhzaT0iaHR0cDovL3d3dy53My5vcmcvMjAwMS9YTUxTY2hlbWEtaW5zdGFuY2UiPjxDYW5FdmFsdWF0ZUZ1dHVyZVBhY2thZ2VzPmZhbHNlPC9DYW5FdmFsdWF0ZUZ1dHVyZVBhY2thZ2VzPjxGaXJld2FsbEVuYWJsZWQ+dHJ1ZTwvRmlyZXdhbGxFbmFibGVkPjwvUGVybWlzc2lvbkxpc3Q+lQEAAAAAAABzAQAAPD94bWwgdmVyc2lvbj0iMS4wIiBlbmNvZGluZz0idXRmLTgiID8+PExvY2FsUGFja2FnZU1ldGFkYXRhRmlsZSB4bWxuczp4c2Q9Imh0dHA6Ly93d3cudzMub3JnLzIwMDEvWE1MU2NoZW1hIiB4bWxuczp4c2k9Imh0dHA6Ly93d3cudzMub3JnLzIwMDEvWE1MU2NoZW1hLWluc3RhbmNlIj48SXRlbXM+PEl0ZW0+PEl0ZW1Mb2NhdGlvbj48SXRlbVR5cGU+QWxsRm9ybXVsYXM8L0l0ZW1UeXBlPjxJdGVtUGF0aCAvPjwvSXRlbUxvY2F0aW9uPjxTdGFibGVFbnRyaWVzPjxFbnRyeSBUeXBlPSJSZWxhdGlvbnNoaXBzIiBWYWx1ZT0ic0FBQUFBQT09IiAvPjwvU3RhYmxlRW50cmllcz48L0l0ZW0+PC9JdGVtcz48L0xvY2FsUGFja2FnZU1ldGFkYXRhRmlsZT4WAAAAUEsFBgAAAAAAAAAAAAAAAAAAAAAAACYBAAABAAAA0Iyd3wEV0RGMegDAT8KX6wEAAABSzpCZZto1RJRGOYJZeOe/AAAAAAIAAAAAABBmAAAAAQAAIAAAABIfzpdhzJLDCA8K31hd93o7UqkFtEKbS9jEOufAambxAAAAAA6AAAAAAgAAIAAAAJbGwjnRHK/9RCm7TpoakUOt4ZFF3gTQqZGuKnlInQvyUAAAAFLA+CZ5f0F06Jn0iX88O687OT6lU0KXr8FKEVB61WzMowbD1IVZ/KQ4D6lpCiZEJDvl/PjGlOSaY6wWVopP8y9uBsFe8RsFgbruLRDnETokQAAAAN6Dk7weKYwFl5YFJrz9XUBSYmh8kJZNfxKVhuZldaZEjyvZ4wuC5ZQFZvyC27B89lx/8Hy8BgoLmU5Y5EdPt8s=</DataMashup>
+<DataMashup xmlns="http://schemas.microsoft.com/DataMashup">AAAAAGwDAABQSwMECgAAAAAAh07iQAAAAAAAAAAAAAAAAAcAAABDb25maWcvUEsDBBQAAAAIAIdO4kASOP6YnwAAAPMAAAASAAAAQ29uZmlnL1BhY2thZ2UueG1shY9NC4IwHMa/iuzuNmdRyN958JoRBNF1zDVHOsPNJn36jDK6dXtefofngWLq2uiuBmd6m6MEUxQpK/vaWJ2j0V/iLSo4HIS8Cq2iGbYum1ydo8b7W0ZICAGHFPeDJozShJyr3VE2qhPoC5v/cGys88JKhTic3mM4w8lqg9N1iimQJYTK2EUzzOa9r/YnhHJs/Tgo/mjicg9ksUA+H/gTUEsDBAoAAAAAAIdO4kAAAAAAAAAAAAAAAAAJAAAARm9ybXVsYXMvUEsDBBQAAAAIAIdO4kAoike4DgAAABEAAAATAAAARm9ybXVsYXMvU2VjdGlvbjEubStOTS7JzM9TCIbQhtYAUEsDBBQAAAAIAIdO4kB/v9PKnQAAAOQAAAATAAAAW0NvbnRlbnRfVHlwZXNdLnhtbG2PSw7CMAxErxJ5n7qwQAg17aJwAy4QBfcjmo8aF4Xbk9AdYunxPM+46ZJdxIvWOHun4FDVIMgZ/5jdqGDjQZ6ha5v7O1AU2eqigok5XBCjmcjqWPlALm8Gv1rNeVxHDNo89Uh4rOsTGu+YHEsuN6BtrjTobWFxS1neYzMOot99JUoBU2IsMv4F7I9dh7DMRnN+ApO0UdoC4rd2+wFQSwECFAAUAAAACACHTuJAf7/Typ0AAADkAAAAEwAAAAAAAAABACAAAABaAQAAW0NvbnRlbnRfVHlwZXNdLnhtbFBLAQIUAAoAAAAAAIdO4kAAAAAAAAAAAAAAAAAHAAAAAAAAAAAAEAAAAAAAAABDb25maWcvUEsBAhQAFAAAAAgAh07iQBI4/pifAAAA8wAAABIAAAAAAAAAAQAgAAAAJQAAAENvbmZpZy9QYWNrYWdlLnhtbFBLAQIUAAoAAAAAAIdO4kAAAAAAAAAAAAAAAAAJAAAAAAAAAAAAEAAAAPQAAABGb3JtdWxhcy9QSwECFAAUAAAACACHTuJAKIpHuA4AAAARAAAAEwAAAAAAAAABACAAAAAbAQAARm9ybXVsYXMvU2VjdGlvbjEubVBLBQYAAAAABQAFAC4BAAAoAgAAAAAOAQAAPD94bWwgdmVyc2lvbj0iMS4wIiBlbmNvZGluZz0idXRmLTgiID8+PFBlcm1pc3Npb25MaXN0IHhtbG5zOnhzZD0iaHR0cDovL3d3dy53My5vcmcvMjAwMS9YTUxTY2hlbWEiIHhtbG5zOnhzaT0iaHR0cDovL3d3dy53My5vcmcvMjAwMS9YTUxTY2hlbWEtaW5zdGFuY2UiPjxDYW5FdmFsdWF0ZUZ1dHVyZVBhY2thZ2VzPmZhbHNlPC9DYW5FdmFsdWF0ZUZ1dHVyZVBhY2thZ2VzPjxGaXJld2FsbEVuYWJsZWQ+dHJ1ZTwvRmlyZXdhbGxFbmFibGVkPjwvUGVybWlzc2lvbkxpc3Q+lQEAAAAAAABzAQAAPD94bWwgdmVyc2lvbj0iMS4wIiBlbmNvZGluZz0idXRmLTgiID8+PExvY2FsUGFja2FnZU1ldGFkYXRhRmlsZSB4bWxuczp4c2Q9Imh0dHA6Ly93d3cudzMub3JnLzIwMDEvWE1MU2NoZW1hIiB4bWxuczp4c2k9Imh0dHA6Ly93d3cudzMub3JnLzIwMDEvWE1MU2NoZW1hLWluc3RhbmNlIj48SXRlbXM+PEl0ZW0+PEl0ZW1Mb2NhdGlvbj48SXRlbVR5cGU+QWxsRm9ybXVsYXM8L0l0ZW1UeXBlPjxJdGVtUGF0aCAvPjwvSXRlbUxvY2F0aW9uPjxTdGFibGVFbnRyaWVzPjxFbnRyeSBUeXBlPSJSZWxhdGlvbnNoaXBzIiBWYWx1ZT0ic0FBQUFBQT09IiAvPjwvU3RhYmxlRW50cmllcz48L0l0ZW0+PC9JdGVtcz48L0xvY2FsUGFja2FnZU1ldGFkYXRhRmlsZT4WAAAAUEsFBgAAAAAAAAAAAAAAAAAAAAAAACYBAAABAAAA0Iyd3wEV0RGMegDAT8KX6wEAAABSzpCZZto1RJRGOYJZeOe/AAAAAAIAAAAAABBmAAAAAQAAIAAAAK4Scs6v6jrJKAuVRCwIQWJn50RkJAlnP72hqVixfrufAAAAAA6AAAAAAgAAIAAAAIDyiakeiqXkOBr6wvcl1adqAtwuZrIg0Mau4Pync11FUAAAABpFEBn0xCjSEs5w54BLnxcIN9xSDRyuNHPFftSH1/+JKgXl5s3EyZkxrdsfFpNlfNysg1oIdc6WgrLiZHqRNfbnBw94krFz4rs7BffZRWs5QAAAAEF54gMsZK/jhCG9h1TgnedqqtnU7Srm8tppELR+1r1xYhXkd2buF7HbHZo1P6HC1bkAsNMO+gUCAgEG7+Rvctw=</DataMashup>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B1689A60-E8A4-4554-84C5-E02241C0F46A}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ECDBB26B-5A60-475F-8CD9-DD98CB833E8A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/DataMashup"/>
   </ds:schemaRefs>

</xml_diff>